<commit_message>
feat: implement loopback HTTP API for local control and transcription
- Add commands for managing the HTTP API status and port settings.
- Create subtitle export helpers for SRT and VTT formats.
- Implement the HTTP API server using Axum for handling transcription requests.
- Introduce a WatchFolderManager for auto-transcribing files in specified directories.
- Develop a settings UI component for enabling and configuring the local API.
</commit_message>
<xml_diff>
--- a/VoxJot_Model_Registry.xlsx
+++ b/VoxJot_Model_Registry.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -101,8 +101,17 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -143,6 +152,16 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
         <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -230,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -322,6 +341,17 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -582,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -643,7 +673,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Whisper (GGML), Parakeet, Moonshine, SenseVoice (ONNX), GigaAM (ONNX), QwenAudio</t>
+          <t>Whisper (GGML), Parakeet, Moonshine, SenseVoice (ONNX), GigaAM (ONNX), QwenAudio, MLX Audio STT</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -653,7 +683,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>14 models incl. 1 coming soon</t>
+          <t>26 models incl. 1 coming soon (Apple Silicon MLX variants on macOS aarch64)</t>
         </is>
       </c>
     </row>
@@ -895,6 +925,18 @@
       <c r="C19" s="28" t="n"/>
       <c r="D19" s="28" t="n"/>
       <c r="E19" s="28" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="33" t="inlineStr">
+        <is>
+          <t>Last updated</t>
+        </is>
+      </c>
+      <c r="B21" s="34" t="inlineStr">
+        <is>
+          <t>2026-04-25 — synced to src-tauri/src/managers/model.rs and src-tauri/src/ollama.rs</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -923,7 +965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1799,6 +1841,690 @@
       <c r="L16" t="inlineStr">
         <is>
           <t>https://huggingface.co/Qwen/Qwen2-Audio-7B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Whisper Tiny</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>tiny</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Full precision</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Whisper (GGML)</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="H17" s="35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I17" s="36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>99 languages (multilingual)</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/ggerganov/whisper.cpp</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Whisper Tiny (English)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>tiny.en</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Full precision (English-only)</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>75</v>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Whisper (GGML)</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="G18" s="13" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H18" s="37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I18" s="36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>English (en)</t>
+        </is>
+      </c>
+      <c r="K18" s="16" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/ggerganov/whisper.cpp</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Whisper Base</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Full precision</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>142</v>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Whisper (GGML)</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="G19" s="13" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="H19" s="35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I19" s="36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>99 languages (multilingual)</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/ggerganov/whisper.cpp</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Whisper Base (English)</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>base.en</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Full precision (English-only)</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>142</v>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Whisper (GGML)</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G20" s="13" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H20" s="37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I20" s="36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>English (en)</t>
+        </is>
+      </c>
+      <c r="K20" s="16" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/ggerganov/whisper.cpp</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Whisper Small (English)</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>small.en</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Full precision (English-only)</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>487</v>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Whisper (GGML)</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G21" s="13" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="H21" s="37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I21" s="36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>English (en)</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/ggerganov/whisper.cpp</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Whisper Medium (English)</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>medium.en</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Full precision (English-only)</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Whisper (GGML)</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="H22" s="37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I22" s="36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>English (en)</t>
+        </is>
+      </c>
+      <c r="K22" s="16" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/ggerganov/whisper.cpp</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Whisper Large V3 Turbo (MLX)</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>mlx-whisper-large-v3-turbo</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>MLX / mlx-audio sidecar</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>MLX Audio STT</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G23" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H23" s="37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I23" s="36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>99 languages (multilingual)</t>
+        </is>
+      </c>
+      <c r="K23" s="16" t="inlineStr">
+        <is>
+          <t>Available ★ Recommended (Apple Silicon)</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/mlx-community/whisper-large-v3-turbo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Distil-Whisper Large V3 (MLX)</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>mlx-distil-whisper-large-v3</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>MLX / mlx-audio sidecar</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>MLX Audio STT</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="H24" s="37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I24" s="36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>English (en)</t>
+        </is>
+      </c>
+      <c r="K24" s="16" t="inlineStr">
+        <is>
+          <t>Available (Apple Silicon)</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/mlx-community/distil-whisper-large-v3</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Qwen3 ASR (MLX)</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>mlx-qwen3-asr</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>MLX / mlx-audio sidecar</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>MLX Audio STT</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G25" s="13" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="H25" s="37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I25" s="36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>zh, en, ja, ko, mul</t>
+        </is>
+      </c>
+      <c r="K25" s="16" t="inlineStr">
+        <is>
+          <t>Available (Apple Silicon)</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/mlx-community</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Parakeet V3 (MLX)</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>mlx-parakeet-v3</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>MLX / mlx-audio sidecar</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>MLX Audio STT</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G26" s="13" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="H26" s="37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I26" s="36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>25 European languages (bg, hr, cs, da, nl, en, et, fi, fr, de, el, hu, it, lv, lt, mt, pl, pt, ro, sk, sl, es, sv, ru, uk)</t>
+        </is>
+      </c>
+      <c r="K26" s="16" t="inlineStr">
+        <is>
+          <t>Available (Apple Silicon)</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/mlx-community/parakeet-tdt-0.6b-v3</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Voxtral Mini 3B (MLX)</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>mlx-voxtral-mini-3b</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>MLX Community / BF16</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>MLX Audio STT</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G27" s="13" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H27" s="37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I27" s="36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>en, fr, de, es, it, pt, nl, hi</t>
+        </is>
+      </c>
+      <c r="K27" s="16" t="inlineStr">
+        <is>
+          <t>Available (Apple Silicon)</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/mlx-community/Voxtral-Mini-3B-2507-bf16</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Voxtral Mini 4B Realtime (MLX)</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>mlx-voxtral-mini-4b-realtime</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>MLX Community / 4-bit</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>MLX Audio STT</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G28" s="13" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="H28" s="37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I28" s="36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>ar, de, en, es, fr, hi, it, nl, pt, zh, ja, ko, ru</t>
+        </is>
+      </c>
+      <c r="K28" s="16" t="inlineStr">
+        <is>
+          <t>Available (Apple Silicon)</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/mlx-community/Voxtral-Mini-4B-Realtime-2602-4bit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: standardize color palette using --muted CSS variable and add new model evaluation documents
</commit_message>
<xml_diff>
--- a/VoxJot_Model_Registry.xlsx
+++ b/VoxJot_Model_Registry.xlsx
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <f>COUNTA('STT Models'!A3:A100)-COUNTBLANK('STT Models'!A3:A100)</f>
+        <f>COUNTA('STT Models'!A3:A100)</f>
         <v/>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -686,15 +686,13 @@
           <t>Whisper (GGML), Parakeet, Moonshine, SenseVoice (ONNX), GigaAM (ONNX), QwenAudio, MLX Audio STT</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>26 models incl. 1 coming soon (Apple Silicon MLX variants on macOS aarch64)</t>
-        </is>
+      <c r="D3" s="3">
+        <f>IF(COUNTIF('STT Models'!J3:J100,"Yes")=0,"None",COUNTIF('STT Models'!J3:J100,"Yes")&amp;" models")</f>
+        <v/>
+      </c>
+      <c r="E3" s="4">
+        <f>B3&amp;" speech-to-text profiles (includes 1 Coming soon · Apple Silicon MLX lines where indicated)."</f>
+        <v/>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1">
@@ -704,7 +702,7 @@
         </is>
       </c>
       <c r="B4" s="6">
-        <f>COUNTA('TTS Models'!A3:A100)-COUNTBLANK('TTS Models'!A3:A100)</f>
+        <f>COUNTA('TTS Models'!A3:A100)</f>
         <v/>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -713,13 +711,12 @@
         </is>
       </c>
       <c r="D4" s="6">
-        <f>COUNTIF('TTS Models'!F3:F100,"Yes")&amp;" models"</f>
+        <f>IF(COUNTIF('TTS Models'!G3:G100,"Yes")=0,"None",COUNTIF('TTS Models'!G3:G100,"Yes")&amp;" models")</f>
         <v/>
       </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Expanded with tested Apple Silicon MLX models that are confirmed working and audible in Vox Jot.</t>
-        </is>
+      <c r="E4" s="7">
+        <f>B4&amp;" text-to-speech profiles (Sherpa-/sidecar/MLX; voice cloning ✓ counted in Voice Cloning column)."</f>
+        <v/>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
@@ -729,7 +726,7 @@
         </is>
       </c>
       <c r="B5" s="3">
-        <f>COUNTA('LLM Models'!A3:A100)-COUNTBLANK('LLM Models'!A3:A100)</f>
+        <f>COUNTA('LLM Models'!A3:A100)</f>
         <v/>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -737,15 +734,13 @@
           <t>Ollama (local inference)</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>22 recommended Ollama models (0.5B–4B range)</t>
-        </is>
+      <c r="D5" s="3">
+        <f>IF(COUNTIF('LLM Models'!H3:H100,"Yes")=0,"None",COUNTIF('LLM Models'!H3:H100,"Yes")&amp;" models")</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>B5&amp;" locally recommended LLM presets (tiny/medium routing via Refine)."</f>
+        <v/>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
@@ -763,10 +758,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>11 TTS models</t>
-        </is>
+      <c r="D6" s="8">
+        <f>IF(SUM(COUNTIF('STT Models'!J3:J100,"Yes"),COUNTIF('TTS Models'!G3:G100,"Yes"),COUNTIF('LLM Models'!H3:H100,"Yes"))=0,"None",SUM(COUNTIF('STT Models'!J3:J100,"Yes"),COUNTIF('TTS Models'!G3:G100,"Yes"),COUNTIF('LLM Models'!H3:H100,"Yes"))&amp;" models")</f>
+        <v/>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
@@ -944,7 +938,7 @@
       </c>
       <c r="B21" s="34" t="inlineStr">
         <is>
-          <t>2026-04-25 — synced to src-tauri/src/managers/model.rs and src-tauri/src/ollama.rs</t>
+          <t>2026-04-27 — registry export; synced to src-tauri/src/managers/model.rs &amp; src-tauri/src/ollama.rs. Summary: COUNTA row counts &amp; Voice Cloning SUM/COUNTIF across STT/J, TTS/G, LLM/H.</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1437,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>https://huggingface.co/nvidia/parakeet-tdt-0.6b-v3</t>
+          <t>https://huggingface.co/nvidia/parakeet-tdt-0.6b-v2</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2298,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2322,11 +2316,7 @@
           <t>MLX / mlx-audio sidecar</t>
         </is>
       </c>
-      <c r="E23" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E23" s="12" t="n"/>
       <c r="F23" s="3" t="inlineStr">
         <is>
           <t>MLX Audio STT</t>
@@ -2367,7 +2357,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2385,11 +2375,7 @@
           <t>MLX / mlx-audio sidecar</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E24" s="12" t="n"/>
       <c r="F24" s="3" t="inlineStr">
         <is>
           <t>MLX Audio STT</t>
@@ -2430,7 +2416,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2448,11 +2434,7 @@
           <t>MLX / mlx-audio sidecar</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E25" s="12" t="n"/>
       <c r="F25" s="3" t="inlineStr">
         <is>
           <t>MLX Audio STT</t>
@@ -2493,7 +2475,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2511,11 +2493,7 @@
           <t>MLX / mlx-audio sidecar</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E26" s="12" t="n"/>
       <c r="F26" s="3" t="inlineStr">
         <is>
           <t>MLX Audio STT</t>
@@ -2556,7 +2534,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -2574,11 +2552,7 @@
           <t>MLX Community / BF16</t>
         </is>
       </c>
-      <c r="E27" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E27" s="12" t="n"/>
       <c r="F27" s="3" t="inlineStr">
         <is>
           <t>MLX Audio STT</t>
@@ -2619,7 +2593,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -2637,11 +2611,7 @@
           <t>MLX Community / 4-bit</t>
         </is>
       </c>
-      <c r="E28" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E28" s="12" t="n"/>
       <c r="F28" s="3" t="inlineStr">
         <is>
           <t>MLX Audio STT</t>
@@ -3862,7 +3832,7 @@
     <row r="22" ht="18" customHeight="1">
       <c r="A22" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3887,7 +3857,7 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>372 MB | Tested + audible on Mac ✅</t>
+          <t>372 MB · Tested + audible on Mac ✅</t>
         </is>
       </c>
       <c r="G22" s="15" t="inlineStr">
@@ -3919,7 +3889,7 @@
     <row r="23" ht="18" customHeight="1">
       <c r="A23" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3944,7 +3914,7 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>2.4 GB | Tested + audible on Mac ✅</t>
+          <t>2.4 GB · Tested + audible on Mac ✅</t>
         </is>
       </c>
       <c r="G23" s="15" t="inlineStr">
@@ -3976,7 +3946,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4001,7 +3971,7 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>2.3 GB | Tested + audible on Mac ✅</t>
+          <t>2.3 GB · Tested + audible on Mac ✅</t>
         </is>
       </c>
       <c r="G24" s="15" t="inlineStr">
@@ -4033,7 +4003,7 @@
     <row r="25" ht="18" customHeight="1">
       <c r="A25" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4058,7 +4028,7 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>4.2 GB | Tested + audible on Mac ✅</t>
+          <t>4.2 GB · Tested + audible on Mac ✅</t>
         </is>
       </c>
       <c r="G25" s="15" t="inlineStr">
@@ -4090,7 +4060,7 @@
     <row r="26" ht="18" customHeight="1">
       <c r="A26" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -4115,7 +4085,7 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>3.0 GB | Tested + audible on Mac ✅</t>
+          <t>3.0 GB · Tested + audible on Mac ✅</t>
         </is>
       </c>
       <c r="G26" s="15" t="inlineStr">
@@ -4147,7 +4117,7 @@
     <row r="27" ht="18" customHeight="1">
       <c r="A27" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4172,7 +4142,7 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>2.7 GB | Tested + audible on Mac ✅</t>
+          <t>2.7 GB · Tested + audible on Mac ✅</t>
         </is>
       </c>
       <c r="G27" s="15" t="inlineStr">
@@ -4204,7 +4174,7 @@
     <row r="28" ht="18" customHeight="1">
       <c r="A28" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4229,7 +4199,7 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>5.8 GB | Tested + audible on Mac ✅ | Requires reference audio for current working flow</t>
+          <t>5.8 GB · Tested + audible on Mac ✅ · Requires reference audio for current working flow</t>
         </is>
       </c>
       <c r="G28" s="15" t="inlineStr">
@@ -4261,7 +4231,7 @@
     <row r="29" ht="18" customHeight="1">
       <c r="A29" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4286,7 +4256,7 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>837 MB | Tested + audible on Mac ✅</t>
+          <t>837 MB · Tested + audible on Mac ✅</t>
         </is>
       </c>
       <c r="G29" s="15" t="inlineStr">
@@ -4318,7 +4288,7 @@
     <row r="30" ht="18" customHeight="1">
       <c r="A30" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4343,7 +4313,7 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>3.3 GB | Tested + audible on Mac ✅ | 20 preset voices</t>
+          <t>3.3 GB · Tested + audible on Mac ✅ · 20 preset voices</t>
         </is>
       </c>
       <c r="G30" s="15" t="inlineStr">
@@ -4375,7 +4345,7 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" t="inlineStr">
         <is>
-          <t>✅</t>
+          <t>🟢✅</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -4400,7 +4370,7 @@
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>4.3 GB | Tested + audible on Mac ✅ | Requires Llama 3.2 license</t>
+          <t>4.3 GB · Tested + audible on Mac ✅ · Requires Llama 3.2 license</t>
         </is>
       </c>
       <c r="G31" s="15" t="inlineStr">
@@ -4440,42 +4410,42 @@
           <t>Liquid LFM2.5 Audio 1.5B</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>lfm2.5-audio-1.5b-gguf</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>1.5B</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>GGUF · 1.5B</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>GGUF (custom llama-liquid-audio)</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>Unified ASR &amp; TTS</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>1.5B · Unified ASR + TTS (one checkpoint)</t>
+        </is>
+      </c>
+      <c r="G32" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H32" s="15" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I32" s="7" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="J32" s="22" t="inlineStr">
         <is>
           <t>Apple Silicon (GGUF)</t>
         </is>
@@ -4502,42 +4472,42 @@
           <t>VibeVoice Realtime 0.5B</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>vibevoice-realtime-0.5b</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>0.5B</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Realtime · 0.5B</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>Python Sidecar (PyTorch)</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Low-latency TTS</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>0.5B · Low-latency TTS</t>
+        </is>
+      </c>
+      <c r="G33" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H33" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="J33" s="22" t="inlineStr">
         <is>
           <t>Apple Silicon (MPS)</t>
         </is>
@@ -5648,30 +5618,30 @@
           <t>Liquid LFM2 1.2B Tool</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>lfm2-1.2b-tool-gguf</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>1.2B</t>
         </is>
       </c>
-      <c r="E25" t="n">
+      <c r="E25" s="24" t="n">
         <v>0.73</v>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>GGUF (llama.cpp)</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>Optimized for tool calling on edge</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="H25" s="15" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
feat: cross-platform screen OCR, OCR engines hub, and refine models
- Add Linux/Windows screen context OCR modules, ocr_models, tess resources layout
- Scripts to fetch Tesseract binaries/tessdata and HF mirror upload helpers
- Model hub OCR engines section; settings and i18n updates
- Refine models, shortcuts, storage paths, LFM audio GGUF, Moss eval doc

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/VoxJot_Model_Registry.xlsx
+++ b/VoxJot_Model_Registry.xlsx
@@ -969,7 +969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N28"/>
+  <dimension ref="A1:N29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2647,6 +2647,70 @@
         <is>
           <t>https://huggingface.co/mlx-community/Voxtral-Mini-4B-Realtime-2602-4bit</t>
         </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>🔴❌</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>MOSS-Audio-4B-Instruct</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>moss-audio-4b-instruct</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Full precision (FP16/BF16)</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Sidecar / MLX (pending)</t>
+        </is>
+      </c>
+      <c r="G29" s="13" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H29" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I29" s="37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J29" s="36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>en, zh</t>
+        </is>
+      </c>
+      <c r="L29" s="16" t="inlineStr">
+        <is>
+          <t>Skip (CUDA only)</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>https://huggingface.co/OpenMOSS-Team/MOSS-Audio-4B-Instruct</t>
+        </is>
+      </c>
+      <c r="N29" t="n">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>